<commit_message>
TICVAI: leftovers closed, build readiness updated for the evening of 29 September
- P11 Accreditation Web calls the accreditation operations, not the
  approvals placeholders; flow F23 follows. Document verification waits
  on a read of an application's documents (BL-180), recorded as a gap.
- getResourceQualifications bound on BO-857, the resource profile.
- 19 tables no operation reached now have their writers named (50
  lineage references); evaluateAccess returns a consistency token now
  that it writes the authorisation audit.
- Billing-statement reads need ORDER_VIEW for staff.
- Build readiness report, page and both workbooks updated: 98% of
  requirements, the AI design decided (none to the client), what is left.
- tools/applied/leftovers-29-september.py records the edits.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ticvai/handoff/TICVAI_Client_Questions.xlsx
+++ b/ticvai/handoff/TICVAI_Client_Questions.xlsx
@@ -1673,7 +1673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E107"/>
+  <dimension ref="A1:E104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4079,75 +4079,6 @@
       </c>
       <c r="E104" s="4" t="inlineStr"/>
     </row>
-    <row r="105">
-      <c r="A105" s="5" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="B105" s="6" t="inlineStr">
-        <is>
-          <t>P11</t>
-        </is>
-      </c>
-      <c r="C105" s="6" t="inlineStr">
-        <is>
-          <t>ACC-002</t>
-        </is>
-      </c>
-      <c r="D105" s="6" t="inlineStr">
-        <is>
-          <t>Registration Form</t>
-        </is>
-      </c>
-      <c r="E105" s="4" t="inlineStr"/>
-    </row>
-    <row r="106">
-      <c r="A106" s="2" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="B106" s="3" t="inlineStr">
-        <is>
-          <t>P11</t>
-        </is>
-      </c>
-      <c r="C106" s="3" t="inlineStr">
-        <is>
-          <t>ACC-003</t>
-        </is>
-      </c>
-      <c r="D106" s="3" t="inlineStr">
-        <is>
-          <t>Application Review &amp; Submit</t>
-        </is>
-      </c>
-      <c r="E106" s="4" t="inlineStr"/>
-    </row>
-    <row r="107">
-      <c r="A107" s="5" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="B107" s="6" t="inlineStr">
-        <is>
-          <t>P11</t>
-        </is>
-      </c>
-      <c r="C107" s="6" t="inlineStr">
-        <is>
-          <t>ACC-004</t>
-        </is>
-      </c>
-      <c r="D107" s="6" t="inlineStr">
-        <is>
-          <t>Application Status Tracking</t>
-        </is>
-      </c>
-      <c r="E107" s="4" t="inlineStr"/>
-    </row>
   </sheetData>
   <autoFilter ref="A1:E1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
TICVAI: release refresh for r2 (refresh-safe passed on 3dd003aa: JUDGEMENT PASS, no failure outside tools/refresh-safe-baseline.json)
All 65 refresh steps, then 54 checkers, judged against the baseline; derived files,
the forward migrations after r1, the changelog index, plan tasks and the six repos/* mirrors.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ticvai/handoff/TICVAI_Client_Questions.xlsx
+++ b/ticvai/handoff/TICVAI_Client_Questions.xlsx
@@ -936,7 +936,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>They are 0% of the 2668 operations and exactly the ones with no data lineage. Nothing behind them can be built until they are agreed.</t>
+          <t>They are 0% of the 2731 operations and exactly the ones with no data lineage. Nothing behind them can be built until they are agreed.</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -1029,7 +1029,7 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>P09 (1)</t>
+          <t>P08 (1)</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Is the AI Configuration Assistant in this delivery? 0 screens - setup discovery, guided Q&amp;A, blueprint, execution, rollback and audit.</t>
+          <t>Is the AI Configuration Assistant in this delivery? 15 screens - setup discovery, guided Q&amp;A, blueprint, execution, rollback and audit.</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -1102,7 +1102,7 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Is Forecasting in this delivery? 0 screens with no operation behind them.</t>
+          <t>Is Forecasting in this delivery? 1 screens with no operation behind them.</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -1146,12 +1146,12 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Is AI governance in this delivery? 1 screens - capability registry, risk classification, policy builder, approval review.</t>
+          <t>Is AI governance in this delivery? 6 screens - capability registry, risk classification, policy builder, approval review.</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>The ai contract has 31 operations in total, against 1 screens of AI product with nothing behind them.</t>
+          <t>The ai contract has 31 operations in total, against 22 screens of AI product with nothing behind them.</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
@@ -1435,7 +1435,7 @@
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>P09 (1)</t>
+          <t>P08 (1)</t>
         </is>
       </c>
       <c r="H3" s="6" t="inlineStr"/>
@@ -1673,7 +1673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1713,22 +1713,22 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>AI governance and human oversight</t>
+          <t>AI configuration assistant</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>P09</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>ADM-618</t>
+          <t>ADM-121</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Refund Simulator, Risk Analysis &amp; AI Advisor\t126</t>
+          <t>Bulk Product Creation &amp; Catalogue Import</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr"/>
@@ -1736,22 +1736,22 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>AI configuration assistant</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>P02</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>GST-043</t>
+          <t>ADM-242</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>Arabic / RTL Experience</t>
+          <t>Approval Matrix &amp; Multi-Level Approval Configuration</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr"/>
@@ -1759,22 +1759,22 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>AI configuration assistant</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>KSK-001</t>
+          <t>ADM-353</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Attract Loop</t>
+          <t>Webhook Configuration &amp; Subscription Manager</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr"/>
@@ -1782,22 +1782,22 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>AI configuration assistant</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>KSK-014</t>
+          <t>ADM-611</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Out of service</t>
+          <t>Refund Policy &amp; Rule Configuration</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr"/>
@@ -1805,22 +1805,22 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>AI configuration assistant</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>P06</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>EMP-044</t>
+          <t>BO-1161</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Security Rules Testing, Simulation &amp; AI Sandbox</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr"/>
@@ -1828,22 +1828,22 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>AI configuration assistant</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>P06</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>EMP-045</t>
+          <t>BO-1174</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Arabic / RTL</t>
+          <t>Wallet API Catalogue &amp; Endpoint Configuration</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr"/>
@@ -1851,25 +1851,1405 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>AI configuration assistant</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>BO-389</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Reminder &amp; Breach Notification Rules</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>AI configuration assistant</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>BO-390</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Escalation Policy Builder</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>AI configuration assistant</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>BO-403</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Attraction Audit, Dependencies &amp; Governed Actions</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>AI configuration assistant</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>BO-599</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Manual Configuration Center</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>AI configuration assistant</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>BO-646</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Credential Media Configuration</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>AI configuration assistant</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>BO-678</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>Channel, Language &amp; Branding Configuration</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>AI configuration assistant</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>BO-797</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>AI Chatbot Configuration</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>AI configuration assistant</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>BO-817</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>NPS, CSAT &amp; CES Configuration</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>AI configuration assistant</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>P09</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>ADM-408</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Final Package Approval &amp; Handoff</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Forecasting</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>BO-1069</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Platform Health &amp; Observability</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>AI governance and human oversight</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>ADM-618</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Refund Simulator, Risk Analysis &amp; AI Advisor</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>AI governance and human oversight</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>BO-1072</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>Seat Management APIs</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>AI governance and human oversight</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>BO-528</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Dynamic Pricing &amp; AI Recommendation</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>AI governance and human oversight</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>BO-824</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Gamification Command Center</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>AI governance and human oversight</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>BO-841</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Personalization &amp; Localization</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>AI governance and human oversight</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>BO-998</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>Lock Timeout &amp; Concurrency</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>P05</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>KSK-001</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Attract Loop</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>P05</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>KSK-014</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>Out of service</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>EMP-044</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>EMP-045</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>Arabic / RTL</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>ADM-097</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Rule Priority, Conflict Resolution &amp; Dynamic Pricing Test Console</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>ADM-169</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>Buy X Get Y / BOGO Rule Builder</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>ADM-172</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Fixed-Price &amp; “N for X” Offer Builder</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>ADM-173</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>Gift, Free Product &amp; Added-Value Offer Builder</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>ADM-174</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Cross-Category Promotion Builder</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>ADM-199</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>Eligibility Rule Builder</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>ADM-249</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Unified Approval Inbox &amp; Decision Workspace</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>ADM-252</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>SLA, Escalation &amp; Bottleneck Monitor</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>ADM-344</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Digital Signature Management</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>BO-031</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>Asset Register</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>BO-110</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Recipe &amp; BOM Management</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>BO-113</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>Central Kitchen &amp; Commissary Management</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>BO-1133</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>Wallet Usage &amp; Channel Command Center</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>BO-138</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>Production Execution &amp; Batch Management</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>BO-365</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>My Approval Inbox</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>BO-432</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="inlineStr">
+        <is>
+          <t>Real-Time Gameplay Authorization</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>BO-444</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>Redemption Operations Dashboard</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>BO-458</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="inlineStr">
+        <is>
+          <t>Expiry Monitoring &amp; Upcoming Expiration</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>BO-477</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>Reader Command &amp; Event Mapping</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>BO-483</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="inlineStr">
+        <is>
+          <t>Integration Certification &amp; Test Console</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>BO-484</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>Self-Service Experience Command Center</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>BO-587</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Equipment Performance Analytics</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>BO-669</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>Temporary &amp; Seasonal Accreditation</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>BO-674</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>Accreditation Communications Command Center</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>BO-677</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>Communication Template Library</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>BO-679</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="inlineStr">
+        <is>
+          <t>Manual &amp; Bulk Communication Center</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>BO-681</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>Import Validation &amp; Processing Monitor</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>BO-728</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="inlineStr">
+        <is>
+          <t>Outlet Management</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>BO-729</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>Create / Edit Outlet</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>BO-812</t>
+        </is>
+      </c>
+      <c r="D57" s="6" t="inlineStr">
+        <is>
+          <t>Service Recovery</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>BO-822</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>Service Recovery Automation</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>BO-838</t>
+        </is>
+      </c>
+      <c r="D59" s="6" t="inlineStr">
+        <is>
+          <t>Content, Media &amp; Forms</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>BO-942</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>Mobile Operations Control &amp; Offline Sync</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>P09</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="inlineStr">
+        <is>
+          <t>ADM-375</t>
+        </is>
+      </c>
+      <c r="D61" s="6" t="inlineStr">
+        <is>
+          <t>Renewal &amp; Retention Center</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>P09</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>ADM-376</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>Commercial Optimization &amp; Expansion Opportunities</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>P09</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="inlineStr">
+        <is>
+          <t>ADM-379</t>
+        </is>
+      </c>
+      <c r="D63" s="6" t="inlineStr">
+        <is>
+          <t>Welcome &amp; Start Your TICVAI Journey</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>P09</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>ADM-409</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>Purchase / Trial Journey Selection</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>P09</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>ADM-464</t>
+        </is>
+      </c>
+      <c r="D65" s="6" t="inlineStr">
+        <is>
+          <t>Renewal Management Center</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
           <t>P11</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C66" s="3" t="inlineStr">
         <is>
           <t>ACC-001</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D66" s="3" t="inlineStr">
         <is>
           <t>Landing / Programme Overview</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr"/>
+      <c r="E66" s="4" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>P17</t>
+        </is>
+      </c>
+      <c r="C67" s="6" t="inlineStr">
+        <is>
+          <t>SGN-001</t>
+        </is>
+      </c>
+      <c r="D67" s="6" t="inlineStr">
+        <is>
+          <t>Welcome &amp; Start Your TICVAI Journey</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>P17</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>SGN-018</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>Purchase / Trial Journey Selection</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:E1"/>

</xml_diff>

<commit_message>
TICVAI: final refresh for r1 of the fresh start (refresh-safe PASS on 94179670: spec fixes, r1 additions, Block A completeness at 6 tasks a day with the AI cut to A2, AI residency enforcement, venue-map import, flow briefs)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ticvai/handoff/TICVAI_Client_Questions.xlsx
+++ b/ticvai/handoff/TICVAI_Client_Questions.xlsx
@@ -936,7 +936,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>They are 0% of the 2738 operations and exactly the ones with no data lineage. Nothing behind them can be built until they are agreed.</t>
+          <t>They are 0% of the 2758 operations and exactly the ones with no data lineage. Nothing behind them can be built until they are agreed.</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -1673,7 +1673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E68"/>
+  <dimension ref="A1:E66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2224,17 +2224,17 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>P06</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>KSK-001</t>
+          <t>EMP-044</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Attract Loop</t>
+          <t>Accessibility</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr"/>
@@ -2247,17 +2247,17 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>P06</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>KSK-014</t>
+          <t>EMP-045</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Out of service</t>
+          <t>Arabic / RTL</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr"/>
@@ -2270,17 +2270,17 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>P06</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>EMP-044</t>
+          <t>ADM-097</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Rule Priority, Conflict Resolution &amp; Dynamic Pricing Test Console</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr"/>
@@ -2293,17 +2293,17 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>P06</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>EMP-045</t>
+          <t>ADM-169</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>Arabic / RTL</t>
+          <t>Buy X Get Y / BOGO Rule Builder</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr"/>
@@ -2321,12 +2321,12 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>ADM-097</t>
+          <t>ADM-172</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Rule Priority, Conflict Resolution &amp; Dynamic Pricing Test Console</t>
+          <t>Fixed-Price &amp; “N for X” Offer Builder</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr"/>
@@ -2344,12 +2344,12 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>ADM-169</t>
+          <t>ADM-173</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>Buy X Get Y / BOGO Rule Builder</t>
+          <t>Gift, Free Product &amp; Added-Value Offer Builder</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr"/>
@@ -2367,12 +2367,12 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>ADM-172</t>
+          <t>ADM-174</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Fixed-Price &amp; “N for X” Offer Builder</t>
+          <t>Cross-Category Promotion Builder</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr"/>
@@ -2390,12 +2390,12 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>ADM-173</t>
+          <t>ADM-199</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>Gift, Free Product &amp; Added-Value Offer Builder</t>
+          <t>Eligibility Rule Builder</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr"/>
@@ -2413,12 +2413,12 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>ADM-174</t>
+          <t>ADM-249</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Cross-Category Promotion Builder</t>
+          <t>Unified Approval Inbox &amp; Decision Workspace</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr"/>
@@ -2436,12 +2436,12 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>ADM-199</t>
+          <t>ADM-252</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>Eligibility Rule Builder</t>
+          <t>SLA, Escalation &amp; Bottleneck Monitor</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr"/>
@@ -2459,12 +2459,12 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>ADM-249</t>
+          <t>ADM-344</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Unified Approval Inbox &amp; Decision Workspace</t>
+          <t>Digital Signature Management</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr"/>
@@ -2482,12 +2482,12 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>ADM-252</t>
+          <t>BO-031</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>SLA, Escalation &amp; Bottleneck Monitor</t>
+          <t>Asset Register</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr"/>
@@ -2505,12 +2505,12 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>ADM-344</t>
+          <t>BO-110</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Digital Signature Management</t>
+          <t>Recipe &amp; BOM Management</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr"/>
@@ -2528,12 +2528,12 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>BO-031</t>
+          <t>BO-113</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>Asset Register</t>
+          <t>Central Kitchen &amp; Commissary Management</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr"/>
@@ -2551,12 +2551,12 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>BO-110</t>
+          <t>BO-1133</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Recipe &amp; BOM Management</t>
+          <t>Wallet Usage &amp; Channel Command Center</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr"/>
@@ -2574,12 +2574,12 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>BO-113</t>
+          <t>BO-138</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>Central Kitchen &amp; Commissary Management</t>
+          <t>Production Execution &amp; Batch Management</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr"/>
@@ -2597,12 +2597,12 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>BO-1133</t>
+          <t>BO-365</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Wallet Usage &amp; Channel Command Center</t>
+          <t>My Approval Inbox</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr"/>
@@ -2620,12 +2620,12 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>BO-138</t>
+          <t>BO-432</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>Production Execution &amp; Batch Management</t>
+          <t>Real-Time Gameplay Authorization</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr"/>
@@ -2643,12 +2643,12 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>BO-365</t>
+          <t>BO-444</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>My Approval Inbox</t>
+          <t>Redemption Operations Dashboard</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr"/>
@@ -2666,12 +2666,12 @@
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>BO-432</t>
+          <t>BO-458</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>Real-Time Gameplay Authorization</t>
+          <t>Expiry Monitoring &amp; Upcoming Expiration</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr"/>
@@ -2689,12 +2689,12 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>BO-444</t>
+          <t>BO-477</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Redemption Operations Dashboard</t>
+          <t>Reader Command &amp; Event Mapping</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr"/>
@@ -2712,12 +2712,12 @@
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>BO-458</t>
+          <t>BO-483</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>Expiry Monitoring &amp; Upcoming Expiration</t>
+          <t>Integration Certification &amp; Test Console</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr"/>
@@ -2735,12 +2735,12 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>BO-477</t>
+          <t>BO-484</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Reader Command &amp; Event Mapping</t>
+          <t>Self-Service Experience Command Center</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr"/>
@@ -2758,12 +2758,12 @@
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>BO-483</t>
+          <t>BO-587</t>
         </is>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>Integration Certification &amp; Test Console</t>
+          <t>Inventory &amp; Equipment Performance Analytics</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr"/>
@@ -2781,12 +2781,12 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>BO-484</t>
+          <t>BO-669</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Self-Service Experience Command Center</t>
+          <t>Temporary &amp; Seasonal Accreditation</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr"/>
@@ -2804,12 +2804,12 @@
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>BO-587</t>
+          <t>BO-674</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>Inventory &amp; Equipment Performance Analytics</t>
+          <t>Accreditation Communications Command Center</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr"/>
@@ -2827,12 +2827,12 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>BO-669</t>
+          <t>BO-677</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>Temporary &amp; Seasonal Accreditation</t>
+          <t>Communication Template Library</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr"/>
@@ -2850,12 +2850,12 @@
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>BO-674</t>
+          <t>BO-679</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>Accreditation Communications Command Center</t>
+          <t>Manual &amp; Bulk Communication Center</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr"/>
@@ -2873,12 +2873,12 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>BO-677</t>
+          <t>BO-681</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Communication Template Library</t>
+          <t>Import Validation &amp; Processing Monitor</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr"/>
@@ -2896,12 +2896,12 @@
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>BO-679</t>
+          <t>BO-728</t>
         </is>
       </c>
       <c r="D53" s="6" t="inlineStr">
         <is>
-          <t>Manual &amp; Bulk Communication Center</t>
+          <t>Outlet Management</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr"/>
@@ -2919,12 +2919,12 @@
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>BO-681</t>
+          <t>BO-729</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>Import Validation &amp; Processing Monitor</t>
+          <t>Create / Edit Outlet</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr"/>
@@ -2942,12 +2942,12 @@
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>BO-728</t>
+          <t>BO-812</t>
         </is>
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>Outlet Management</t>
+          <t>Service Recovery</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr"/>
@@ -2965,12 +2965,12 @@
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>BO-729</t>
+          <t>BO-822</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>Create / Edit Outlet</t>
+          <t>Service Recovery Automation</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr"/>
@@ -2988,12 +2988,12 @@
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>BO-812</t>
+          <t>BO-838</t>
         </is>
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>Service Recovery</t>
+          <t>Content, Media &amp; Forms</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr"/>
@@ -3011,12 +3011,12 @@
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>BO-822</t>
+          <t>BO-942</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Service Recovery Automation</t>
+          <t>Mobile Operations Control &amp; Offline Sync</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr"/>
@@ -3029,17 +3029,17 @@
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>P08</t>
+          <t>P09</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>BO-838</t>
+          <t>ADM-375</t>
         </is>
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>Content, Media &amp; Forms</t>
+          <t>Renewal &amp; Retention Center</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr"/>
@@ -3052,17 +3052,17 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>P08</t>
+          <t>P09</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>BO-942</t>
+          <t>ADM-376</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Mobile Operations Control &amp; Offline Sync</t>
+          <t>Commercial Optimization &amp; Expansion Opportunities</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr"/>
@@ -3080,12 +3080,12 @@
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>ADM-375</t>
+          <t>ADM-379</t>
         </is>
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>Renewal &amp; Retention Center</t>
+          <t>Welcome &amp; Start Your TICVAI Journey</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr"/>
@@ -3103,12 +3103,12 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>ADM-376</t>
+          <t>ADM-409</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Commercial Optimization &amp; Expansion Opportunities</t>
+          <t>Purchase / Trial Journey Selection</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr"/>
@@ -3126,12 +3126,12 @@
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>ADM-379</t>
+          <t>ADM-464</t>
         </is>
       </c>
       <c r="D63" s="6" t="inlineStr">
         <is>
-          <t>Welcome &amp; Start Your TICVAI Journey</t>
+          <t>Renewal Management Center</t>
         </is>
       </c>
       <c r="E63" s="4" t="inlineStr"/>
@@ -3144,17 +3144,17 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>P09</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>ADM-409</t>
+          <t>ACC-001</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Purchase / Trial Journey Selection</t>
+          <t>Landing / Programme Overview</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr"/>
@@ -3167,17 +3167,17 @@
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>P09</t>
+          <t>P17</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>ADM-464</t>
+          <t>SGN-001</t>
         </is>
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>Renewal Management Center</t>
+          <t>Welcome &amp; Start Your TICVAI Journey</t>
         </is>
       </c>
       <c r="E65" s="4" t="inlineStr"/>
@@ -3190,66 +3190,20 @@
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P17</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>ACC-001</t>
+          <t>SGN-018</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Landing / Programme Overview</t>
+          <t>Purchase / Trial Journey Selection</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="5" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="B67" s="6" t="inlineStr">
-        <is>
-          <t>P17</t>
-        </is>
-      </c>
-      <c r="C67" s="6" t="inlineStr">
-        <is>
-          <t>SGN-001</t>
-        </is>
-      </c>
-      <c r="D67" s="6" t="inlineStr">
-        <is>
-          <t>Welcome &amp; Start Your TICVAI Journey</t>
-        </is>
-      </c>
-      <c r="E67" s="4" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="2" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="B68" s="3" t="inlineStr">
-        <is>
-          <t>P17</t>
-        </is>
-      </c>
-      <c r="C68" s="3" t="inlineStr">
-        <is>
-          <t>SGN-018</t>
-        </is>
-      </c>
-      <c r="D68" s="3" t="inlineStr">
-        <is>
-          <t>Purchase / Trial Journey Selection</t>
-        </is>
-      </c>
-      <c r="E68" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:E1"/>

</xml_diff>

<commit_message>
TICVAI: release refresh for r1 (refresh-safe PASS on 0faecf6e: Sprint 1-2 fix round, AI phase 1/2, refresh speed-up)
refresh-safe on 0faecf6e: 65 of 65 steps, 67 checkers, 0 gate failures, judged PASS against
tools/refresh-safe-baseline.json (check-package 2 known, check-authored-inputs 7 known);
32m34s (derive 27m02s, checks 3m47s). Carries the Sprint 1-2 fix round (FXC, FXP, FXS, RFM),
the AI engine phase split (AIPH-001/002) and the refresh speed-up (RSPD-001).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ticvai/handoff/TICVAI_Client_Questions.xlsx
+++ b/ticvai/handoff/TICVAI_Client_Questions.xlsx
@@ -936,7 +936,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>They are 0% of the 2758 operations and exactly the ones with no data lineage. Nothing behind them can be built until they are agreed.</t>
+          <t>They are 0% of the 2776 operations and exactly the ones with no data lineage. Nothing behind them can be built until they are agreed.</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -1673,7 +1673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E66"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2781,12 +2781,12 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>BO-669</t>
+          <t>BO-674</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Temporary &amp; Seasonal Accreditation</t>
+          <t>Accreditation Communications Command Center</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr"/>
@@ -2804,12 +2804,12 @@
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>BO-674</t>
+          <t>BO-677</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>Accreditation Communications Command Center</t>
+          <t>Communication Template Library</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr"/>
@@ -2827,12 +2827,12 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>BO-677</t>
+          <t>BO-679</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>Communication Template Library</t>
+          <t>Manual &amp; Bulk Communication Center</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr"/>
@@ -2850,12 +2850,12 @@
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>BO-679</t>
+          <t>BO-681</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>Manual &amp; Bulk Communication Center</t>
+          <t>Import Validation &amp; Processing Monitor</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr"/>
@@ -2873,12 +2873,12 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>BO-681</t>
+          <t>BO-728</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Import Validation &amp; Processing Monitor</t>
+          <t>Outlet Management</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr"/>
@@ -2896,12 +2896,12 @@
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>BO-728</t>
+          <t>BO-729</t>
         </is>
       </c>
       <c r="D53" s="6" t="inlineStr">
         <is>
-          <t>Outlet Management</t>
+          <t>Create / Edit Outlet</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr"/>
@@ -2919,12 +2919,12 @@
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>BO-729</t>
+          <t>BO-812</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>Create / Edit Outlet</t>
+          <t>Service Recovery</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr"/>
@@ -2942,12 +2942,12 @@
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>BO-812</t>
+          <t>BO-822</t>
         </is>
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>Service Recovery</t>
+          <t>Service Recovery Automation</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr"/>
@@ -2965,12 +2965,12 @@
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>BO-822</t>
+          <t>BO-838</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>Service Recovery Automation</t>
+          <t>Content, Media &amp; Forms</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr"/>
@@ -2988,12 +2988,12 @@
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>BO-838</t>
+          <t>BO-942</t>
         </is>
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>Content, Media &amp; Forms</t>
+          <t>Mobile Operations Control &amp; Offline Sync</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr"/>
@@ -3006,17 +3006,17 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>P08</t>
+          <t>P09</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>BO-942</t>
+          <t>ADM-375</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Mobile Operations Control &amp; Offline Sync</t>
+          <t>Renewal &amp; Retention Center</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr"/>
@@ -3034,12 +3034,12 @@
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>ADM-375</t>
+          <t>ADM-376</t>
         </is>
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>Renewal &amp; Retention Center</t>
+          <t>Commercial Optimization &amp; Expansion Opportunities</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr"/>
@@ -3057,12 +3057,12 @@
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>ADM-376</t>
+          <t>ADM-379</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Commercial Optimization &amp; Expansion Opportunities</t>
+          <t>Welcome &amp; Start Your TICVAI Journey</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr"/>
@@ -3080,12 +3080,12 @@
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>ADM-379</t>
+          <t>ADM-409</t>
         </is>
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>Welcome &amp; Start Your TICVAI Journey</t>
+          <t>Purchase / Trial Journey Selection</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr"/>
@@ -3103,12 +3103,12 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>ADM-409</t>
+          <t>ADM-464</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Purchase / Trial Journey Selection</t>
+          <t>Renewal Management Center</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr"/>
@@ -3121,17 +3121,17 @@
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>P09</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>ADM-464</t>
+          <t>ACC-001</t>
         </is>
       </c>
       <c r="D63" s="6" t="inlineStr">
         <is>
-          <t>Renewal Management Center</t>
+          <t>Landing / Programme Overview</t>
         </is>
       </c>
       <c r="E63" s="4" t="inlineStr"/>
@@ -3144,17 +3144,17 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P17</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>ACC-001</t>
+          <t>SGN-001</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Landing / Programme Overview</t>
+          <t>Welcome &amp; Start Your TICVAI Journey</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr"/>
@@ -3172,38 +3172,15 @@
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>SGN-001</t>
+          <t>SGN-018</t>
         </is>
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>Welcome &amp; Start Your TICVAI Journey</t>
+          <t>Purchase / Trial Journey Selection</t>
         </is>
       </c>
       <c r="E65" s="4" t="inlineStr"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="2" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="B66" s="3" t="inlineStr">
-        <is>
-          <t>P17</t>
-        </is>
-      </c>
-      <c r="C66" s="3" t="inlineStr">
-        <is>
-          <t>SGN-018</t>
-        </is>
-      </c>
-      <c r="D66" s="3" t="inlineStr">
-        <is>
-          <t>Purchase / Trial Journey Selection</t>
-        </is>
-      </c>
-      <c r="E66" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:E1"/>

</xml_diff>

<commit_message>
r6 gate 1, derived: the full derive of c0a154d1 plus adam-links and the cross-deployable writes table; base for the gate fix round, not a release
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ticvai/handoff/TICVAI_Client_Questions.xlsx
+++ b/ticvai/handoff/TICVAI_Client_Questions.xlsx
@@ -936,7 +936,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>They are 0% of the 2802 operations and exactly the ones with no data lineage. Nothing behind them can be built until they are agreed.</t>
+          <t>They are 0% of the 2804 operations and exactly the ones with no data lineage. Nothing behind them can be built until they are agreed.</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -1673,7 +1673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E65"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3011,12 +3011,12 @@
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>ADM-375</t>
+          <t>ADM-379</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Renewal &amp; Retention Center</t>
+          <t>Welcome &amp; Start Your TICVAI Journey</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr"/>
@@ -3034,12 +3034,12 @@
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>ADM-376</t>
+          <t>ADM-409</t>
         </is>
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>Commercial Optimization &amp; Expansion Opportunities</t>
+          <t>Purchase / Trial Journey Selection</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr"/>
@@ -3052,17 +3052,17 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>P09</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>ADM-379</t>
+          <t>ACC-001</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Welcome &amp; Start Your TICVAI Journey</t>
+          <t>Landing / Programme Overview</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr"/>
@@ -3075,17 +3075,17 @@
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>P09</t>
+          <t>P17</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>ADM-409</t>
+          <t>SGN-001</t>
         </is>
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>Purchase / Trial Journey Selection</t>
+          <t>Welcome &amp; Start Your TICVAI Journey</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr"/>
@@ -3098,89 +3098,20 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>P09</t>
+          <t>P17</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>ADM-464</t>
+          <t>SGN-018</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Renewal Management Center</t>
+          <t>Purchase / Trial Journey Selection</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="5" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="B63" s="6" t="inlineStr">
-        <is>
-          <t>P11</t>
-        </is>
-      </c>
-      <c r="C63" s="6" t="inlineStr">
-        <is>
-          <t>ACC-001</t>
-        </is>
-      </c>
-      <c r="D63" s="6" t="inlineStr">
-        <is>
-          <t>Landing / Programme Overview</t>
-        </is>
-      </c>
-      <c r="E63" s="4" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="B64" s="3" t="inlineStr">
-        <is>
-          <t>P17</t>
-        </is>
-      </c>
-      <c r="C64" s="3" t="inlineStr">
-        <is>
-          <t>SGN-001</t>
-        </is>
-      </c>
-      <c r="D64" s="3" t="inlineStr">
-        <is>
-          <t>Welcome &amp; Start Your TICVAI Journey</t>
-        </is>
-      </c>
-      <c r="E64" s="4" t="inlineStr"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="5" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="B65" s="6" t="inlineStr">
-        <is>
-          <t>P17</t>
-        </is>
-      </c>
-      <c r="C65" s="6" t="inlineStr">
-        <is>
-          <t>SGN-018</t>
-        </is>
-      </c>
-      <c r="D65" s="6" t="inlineStr">
-        <is>
-          <t>Purchase / Trial Journey Selection</t>
-        </is>
-      </c>
-      <c r="E65" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:E1"/>

</xml_diff>

<commit_message>
r8, derived: the full derive of 18658ed9 (every r8 lane, the gate fixes, the guest AI erasure), from the refresh-safe run 20261020-174xxx (D:/wt/refresh-rehearsal/w94, 70 of 70 steps, 25 min); new forward migrations tenant and control V0108 and V0109 (names). Gate judged 7, all expected: started-ticket acknowledgements (the lead's) and ticket links (adam-links.py after this commit)
CHG-exempt: release refresh commit (derived output only; contracts changed only in their generated x-ticvai-consumed-by and screen-count annotations)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ticvai/handoff/TICVAI_Client_Questions.xlsx
+++ b/ticvai/handoff/TICVAI_Client_Questions.xlsx
@@ -936,7 +936,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>They are 0% of the 2804 operations and exactly the ones with no data lineage. Nothing behind them can be built until they are agreed.</t>
+          <t>They are 0% of the 2844 operations and exactly the ones with no data lineage. Nothing behind them can be built until they are agreed.</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -1673,7 +1673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3113,6 +3113,52 @@
       </c>
       <c r="E62" s="4" t="inlineStr"/>
     </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>P17</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="inlineStr">
+        <is>
+          <t>SGN-019</t>
+        </is>
+      </c>
+      <c r="D63" s="6" t="inlineStr">
+        <is>
+          <t>Contract &amp; Billing Cycle Selection</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>P17</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>SGN-024</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>Subscription Confirmation &amp; Commercial Activation</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:E1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
r11, derived: the full derive of 07529eb7 (refresh-safe run 20261029-205644-65140, 72 of 72 steps; gate PASS, 85 checks), with the forward migrations V0118/V0119 for every r11 change
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ticvai/handoff/TICVAI_Client_Questions.xlsx
+++ b/ticvai/handoff/TICVAI_Client_Questions.xlsx
@@ -936,7 +936,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>They are 0% of the 2856 operations and exactly the ones with no data lineage. Nothing behind them can be built until they are agreed.</t>
+          <t>They are 0% of the 2857 operations and exactly the ones with no data lineage. Nothing behind them can be built until they are agreed.</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Is the AI Configuration Assistant in this delivery? 15 screens - setup discovery, guided Q&amp;A, blueprint, execution, rollback and audit.</t>
+          <t>Is the AI Configuration Assistant in this delivery? 17 screens - setup discovery, guided Q&amp;A, blueprint, execution, rollback and audit.</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -1151,7 +1151,7 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>The ai contract has 31 operations in total, against 22 screens of AI product with nothing behind them.</t>
+          <t>The ai contract has 31 operations in total, against 24 screens of AI product with nothing behind them.</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
@@ -1673,7 +1673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E64"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1953,12 +1953,12 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>BO-646</t>
+          <t>BO-602</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Credential Media Configuration</t>
+          <t>POS, Payment &amp; Access Setup</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr"/>
@@ -1976,12 +1976,12 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>BO-678</t>
+          <t>BO-646</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Channel, Language &amp; Branding Configuration</t>
+          <t>Credential Media Configuration</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr"/>
@@ -1999,12 +1999,12 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>BO-797</t>
+          <t>BO-678</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>AI Chatbot Configuration</t>
+          <t>Channel, Language &amp; Branding Configuration</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr"/>
@@ -2022,12 +2022,12 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>BO-817</t>
+          <t>BO-797</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>NPS, CSAT &amp; CES Configuration</t>
+          <t>AI Chatbot Configuration</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr"/>
@@ -2040,17 +2040,17 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>P09</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>ADM-408</t>
+          <t>BO-817</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Final Package Approval &amp; Handoff</t>
+          <t>NPS, CSAT &amp; CES Configuration</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr"/>
@@ -2058,7 +2058,7 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Forecasting</t>
+          <t>AI configuration assistant</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
@@ -2068,12 +2068,12 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>BO-1069</t>
+          <t>BO-836</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>Platform Health &amp; Observability</t>
+          <t>Design System &amp; Components</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr"/>
@@ -2081,22 +2081,22 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>AI governance and human oversight</t>
+          <t>AI configuration assistant</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>P08</t>
+          <t>P09</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>ADM-618</t>
+          <t>ADM-408</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Refund Simulator, Risk Analysis &amp; AI Advisor</t>
+          <t>Final Package Approval &amp; Handoff</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr"/>
@@ -2104,7 +2104,7 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>AI governance and human oversight</t>
+          <t>Forecasting</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
@@ -2114,12 +2114,12 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>BO-1072</t>
+          <t>BO-1069</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Seat Management APIs</t>
+          <t>Platform Health &amp; Observability</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr"/>
@@ -2137,12 +2137,12 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>BO-528</t>
+          <t>ADM-618</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Dynamic Pricing &amp; AI Recommendation</t>
+          <t>Refund Simulator, Risk Analysis &amp; AI Advisor</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr"/>
@@ -2160,12 +2160,12 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>BO-824</t>
+          <t>BO-1072</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Gamification Command Center</t>
+          <t>Seat Management APIs</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr"/>
@@ -2183,12 +2183,12 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>BO-841</t>
+          <t>BO-528</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Personalization &amp; Localization</t>
+          <t>Dynamic Pricing &amp; AI Recommendation</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr"/>
@@ -2206,12 +2206,12 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>BO-998</t>
+          <t>BO-824</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Lock Timeout &amp; Concurrency</t>
+          <t>Gamification Command Center</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr"/>
@@ -2219,22 +2219,22 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>AI governance and human oversight</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>P06</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>EMP-044</t>
+          <t>BO-841</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Personalization &amp; Localization</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr"/>
@@ -2242,22 +2242,22 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>AI governance and human oversight</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>P06</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>EMP-045</t>
+          <t>BO-998</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Arabic / RTL</t>
+          <t>Lock Timeout &amp; Concurrency</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr"/>
@@ -2270,17 +2270,17 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>P08</t>
+          <t>P06</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>ADM-097</t>
+          <t>EMP-044</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Rule Priority, Conflict Resolution &amp; Dynamic Pricing Test Console</t>
+          <t>Accessibility</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr"/>
@@ -2293,17 +2293,17 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>P08</t>
+          <t>P06</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>ADM-169</t>
+          <t>EMP-045</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>Buy X Get Y / BOGO Rule Builder</t>
+          <t>Arabic / RTL</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr"/>
@@ -2321,12 +2321,12 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>ADM-172</t>
+          <t>ADM-097</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Fixed-Price &amp; “N for X” Offer Builder</t>
+          <t>Rule Priority, Conflict Resolution &amp; Dynamic Pricing Test Console</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr"/>
@@ -2344,12 +2344,12 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>ADM-173</t>
+          <t>ADM-169</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>Gift, Free Product &amp; Added-Value Offer Builder</t>
+          <t>Buy X Get Y / BOGO Rule Builder</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr"/>
@@ -2367,12 +2367,12 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>ADM-174</t>
+          <t>ADM-172</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Cross-Category Promotion Builder</t>
+          <t>Fixed-Price &amp; “N for X” Offer Builder</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr"/>
@@ -2390,12 +2390,12 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>ADM-199</t>
+          <t>ADM-173</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>Eligibility Rule Builder</t>
+          <t>Gift, Free Product &amp; Added-Value Offer Builder</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr"/>
@@ -2413,12 +2413,12 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>ADM-249</t>
+          <t>ADM-174</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Unified Approval Inbox &amp; Decision Workspace</t>
+          <t>Cross-Category Promotion Builder</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr"/>
@@ -2436,12 +2436,12 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>ADM-252</t>
+          <t>ADM-199</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>SLA, Escalation &amp; Bottleneck Monitor</t>
+          <t>Eligibility Rule Builder</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr"/>
@@ -2459,12 +2459,12 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>ADM-344</t>
+          <t>ADM-249</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Digital Signature Management</t>
+          <t>Unified Approval Inbox &amp; Decision Workspace</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr"/>
@@ -2482,12 +2482,12 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>BO-031</t>
+          <t>ADM-252</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>Asset Register</t>
+          <t>SLA, Escalation &amp; Bottleneck Monitor</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr"/>
@@ -2505,12 +2505,12 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>BO-110</t>
+          <t>ADM-344</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Recipe &amp; BOM Management</t>
+          <t>Digital Signature Management</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr"/>
@@ -2528,12 +2528,12 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>BO-113</t>
+          <t>ADM-612</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>Central Kitchen &amp; Commissary Management</t>
+          <t>Refund Allocation &amp; Original Tender Manager</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr"/>
@@ -2551,12 +2551,12 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>BO-1133</t>
+          <t>BO-031</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Wallet Usage &amp; Channel Command Center</t>
+          <t>Asset Register</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr"/>
@@ -2574,12 +2574,12 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>BO-138</t>
+          <t>BO-110</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>Production Execution &amp; Batch Management</t>
+          <t>Recipe &amp; BOM Management</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr"/>
@@ -2597,12 +2597,12 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>BO-365</t>
+          <t>BO-113</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>My Approval Inbox</t>
+          <t>Central Kitchen &amp; Commissary Management</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr"/>
@@ -2620,12 +2620,12 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>BO-432</t>
+          <t>BO-1133</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>Real-Time Gameplay Authorization</t>
+          <t>Wallet Usage &amp; Channel Command Center</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr"/>
@@ -2643,12 +2643,12 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>BO-444</t>
+          <t>BO-138</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>Redemption Operations Dashboard</t>
+          <t>Production Execution &amp; Batch Management</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr"/>
@@ -2666,12 +2666,12 @@
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>BO-458</t>
+          <t>BO-365</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>Expiry Monitoring &amp; Upcoming Expiration</t>
+          <t>My Approval Inbox</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr"/>
@@ -2689,12 +2689,12 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>BO-477</t>
+          <t>BO-432</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Reader Command &amp; Event Mapping</t>
+          <t>Real-Time Gameplay Authorization</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr"/>
@@ -2712,12 +2712,12 @@
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>BO-483</t>
+          <t>BO-444</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>Integration Certification &amp; Test Console</t>
+          <t>Redemption Operations Dashboard</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr"/>
@@ -2735,12 +2735,12 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>BO-484</t>
+          <t>BO-458</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Self-Service Experience Command Center</t>
+          <t>Expiry Monitoring &amp; Upcoming Expiration</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr"/>
@@ -2758,12 +2758,12 @@
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>BO-587</t>
+          <t>BO-477</t>
         </is>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>Inventory &amp; Equipment Performance Analytics</t>
+          <t>Reader Command &amp; Event Mapping</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr"/>
@@ -2781,12 +2781,12 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>BO-674</t>
+          <t>BO-483</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Accreditation Communications Command Center</t>
+          <t>Integration Certification &amp; Test Console</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr"/>
@@ -2804,12 +2804,12 @@
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>BO-677</t>
+          <t>BO-484</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>Communication Template Library</t>
+          <t>Self-Service Experience Command Center</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr"/>
@@ -2827,12 +2827,12 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>BO-679</t>
+          <t>BO-587</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>Manual &amp; Bulk Communication Center</t>
+          <t>Inventory &amp; Equipment Performance Analytics</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr"/>
@@ -2850,12 +2850,12 @@
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>BO-681</t>
+          <t>BO-674</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>Import Validation &amp; Processing Monitor</t>
+          <t>Accreditation Communications Command Center</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr"/>
@@ -2873,12 +2873,12 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>BO-728</t>
+          <t>BO-677</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Outlet Management</t>
+          <t>Communication Template Library</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr"/>
@@ -2896,12 +2896,12 @@
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>BO-729</t>
+          <t>BO-679</t>
         </is>
       </c>
       <c r="D53" s="6" t="inlineStr">
         <is>
-          <t>Create / Edit Outlet</t>
+          <t>Manual &amp; Bulk Communication Center</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr"/>
@@ -2919,12 +2919,12 @@
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>BO-812</t>
+          <t>BO-681</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>Service Recovery</t>
+          <t>Import Validation &amp; Processing Monitor</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr"/>
@@ -2942,12 +2942,12 @@
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>BO-822</t>
+          <t>BO-728</t>
         </is>
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>Service Recovery Automation</t>
+          <t>Outlet Management</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr"/>
@@ -2965,12 +2965,12 @@
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>BO-838</t>
+          <t>BO-729</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>Content, Media &amp; Forms</t>
+          <t>Create / Edit Outlet</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr"/>
@@ -2988,12 +2988,12 @@
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>BO-942</t>
+          <t>BO-812</t>
         </is>
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>Mobile Operations Control &amp; Offline Sync</t>
+          <t>Service Recovery</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr"/>
@@ -3006,17 +3006,17 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>P09</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>ADM-379</t>
+          <t>BO-822</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Welcome &amp; Start Your TICVAI Journey</t>
+          <t>Service Recovery Automation</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr"/>
@@ -3029,17 +3029,17 @@
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>P09</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>ADM-409</t>
+          <t>BO-838</t>
         </is>
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>Purchase / Trial Journey Selection</t>
+          <t>Content, Media &amp; Forms</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr"/>
@@ -3052,17 +3052,17 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>ACC-001</t>
+          <t>BO-917</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Landing / Programme Overview</t>
+          <t>Event Staff &amp; Personnel Allocation</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr"/>
@@ -3075,17 +3075,17 @@
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>P17</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>SGN-001</t>
+          <t>BO-942</t>
         </is>
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>Welcome &amp; Start Your TICVAI Journey</t>
+          <t>Mobile Operations Control &amp; Offline Sync</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr"/>
@@ -3098,17 +3098,17 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>P17</t>
+          <t>P09</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>SGN-018</t>
+          <t>ADM-379</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Purchase / Trial Journey Selection</t>
+          <t>Welcome &amp; Start Your TICVAI Journey</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr"/>
@@ -3121,17 +3121,17 @@
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>P17</t>
+          <t>P09</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>SGN-019</t>
+          <t>ADM-409</t>
         </is>
       </c>
       <c r="D63" s="6" t="inlineStr">
         <is>
-          <t>Contract &amp; Billing Cycle Selection</t>
+          <t>Purchase / Trial Journey Selection</t>
         </is>
       </c>
       <c r="E63" s="4" t="inlineStr"/>
@@ -3144,20 +3144,112 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>ACC-001</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>Landing / Programme Overview</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
           <t>P17</t>
         </is>
       </c>
-      <c r="C64" s="3" t="inlineStr">
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>SGN-001</t>
+        </is>
+      </c>
+      <c r="D65" s="6" t="inlineStr">
+        <is>
+          <t>Welcome &amp; Start Your TICVAI Journey</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>P17</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>SGN-018</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>Purchase / Trial Journey Selection</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>P17</t>
+        </is>
+      </c>
+      <c r="C67" s="6" t="inlineStr">
+        <is>
+          <t>SGN-019</t>
+        </is>
+      </c>
+      <c r="D67" s="6" t="inlineStr">
+        <is>
+          <t>Contract &amp; Billing Cycle Selection</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>P17</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
         <is>
           <t>SGN-024</t>
         </is>
       </c>
-      <c r="D64" s="3" t="inlineStr">
+      <c r="D68" s="3" t="inlineStr">
         <is>
           <t>Subscription Confirmation &amp; Commercial Activation</t>
         </is>
       </c>
-      <c r="E64" s="4" t="inlineStr"/>
+      <c r="E68" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:E1"/>

</xml_diff>